<commit_message>
Version 1: staff dashboard and VERSION-1 report
- Staff dashboard (volunteer-app/web/admin/) on the same Apps Script backend
  and Google Sheet, leaders only: overview, attendance fixes, hours report with
  CSV export, volunteers and trainees (add/edit), fundraising, outings,
  overseas trips and house visits.
- Backend: Dashboard, Fundraising, Outings, Trips and Visits .gs files; 11 new
  tabs created by setup(); Dietary Notes trainee column; attendance edit stamps.
- 19 new backend tests (56 total), local demo data for every section, demo
  .xlsx extended with the new tabs, /admin/ served by the local server.
- VERSION-1.md client report; README, user guide, design notes and PROGRESS.md
  updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/volunteer-app/docs/demo-data/MINDS-Volunteer-Demo-Data.xlsx
+++ b/volunteer-app/docs/demo-data/MINDS-Volunteer-Demo-Data.xlsx
@@ -1,23 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trainees" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volunteers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trainee Notes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volunteer Guide" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Trainees" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Volunteers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sessions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bookings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Attendance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Feedback" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Trainee Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Venues" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Projects" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Volunteer Guide" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Fundraisers" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Products" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Orders" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Order Items" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Outings" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Outing Assignments" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Trips" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Trip Participants" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Trip Logistics" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Trip Expenses" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="House Visits" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -498,7 +509,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>A filled-in copy of the volunteer app's Google Sheet: 8 trainees, 9 volunteers and 1 leader, 4 past sessions with attendance and feedback, and 5 upcoming sessions (23 Oct to 20 Nov 2026).</t>
+          <t>A filled-in copy of the volunteer app's Google Sheet: 8 trainees, 9 volunteers and 1 leader, 4 past sessions with attendance and feedback, 5 upcoming sessions (23 Oct to 20 Nov 2026), and sample records for the staff dashboard (fundraising, an outing, an overseas trip and house visits).</t>
         </is>
       </c>
     </row>
@@ -567,35 +578,35 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Trying it as a demo volunteer</t>
+          <t>Staff dashboard tabs (web/admin/)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>The demo people have no app passwords. To use one, register in the app with their email (any new password). You take over that row and see their history.</t>
+          <t>Fundraisers, Products, Orders, Order Items: the "Charity bake sale" with 4 products and 5 orders. Totals are worked out by the app from the product prices.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>aisha.rahman@example.com: 3 past sessions, booked and confirmed for Art &amp; Craft: clay on 23 Oct with Alex Tan Wei Ming.</t>
+          <t>Outings, Outing Assignments: a zoo outing on 28 Oct with 6 trainees, each looked after by a volunteer, in groups and buses.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ben.koh@example.com: 3 past sessions, waiting for a leader to confirm 23 Oct (he will be paired with Bea again).</t>
+          <t>Trips, Trip Participants, Trip Logistics, Trip Expenses: a Bangkok trip (7 to 11 Dec) with 4 trainees, a checklist and 2 expenses. Medical and dietary notes are copied onto the participant row when a trainee is registered.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>isabel.nair@example.com: one walk-in session on 2 Oct, still to give feedback.</t>
+          <t>House Visits: 3 visit records. History is add-only.</t>
         </is>
       </c>
     </row>
@@ -607,17 +618,59 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Trying it as a demo volunteer</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Rules</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>The demo people have no app passwords. To use one, register in the app with their email (any new password). You take over that row and see their history.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>aisha.rahman@example.com: 3 past sessions, booked and confirmed for Art &amp; Craft: clay on 23 Oct with Alex Tan Wei Ming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ben.koh@example.com: 3 past sessions, waiting for a leader to confirm 23 Oct (he will be paired with Bea again).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>isabel.nair@example.com: one walk-in session on 2 Oct, still to give feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Sarah Yeo is the demo leader but has no account. Make yourself the leader instead (setup guide, Part 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Don't rename the tabs or the headers in row 1 (unless you change gas/Config.gs to match). Editing values is fine: the app re-reads the sheet on every request.</t>
         </is>
@@ -960,6 +1013,2147 @@
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>2026-08-20 10:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Cookies, cards and bags made by trainees, sold at the MINDS open house.</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Price (SGD)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Added By</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Added At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>PD-ADFCD451</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate chip cookies (box of 6)</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CB6D8E4</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Pineapple tarts (box of 10)</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CBBC0AF</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Greeting cards (set of 4)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>PD-D742F744</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Handmade tote bag</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Order ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Fundraiser</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Total (SGD)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Taken By</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Taken At</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>OR-8A99BCEC</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Mdm Rachel Lee</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +65 8100 0001</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>2 × Chocolate chip cookies (box of 6), 1 × Handmade tote bag</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>collected</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:20:00</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>OR-53D7A693</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Office pre-order (Level 5)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>office@example.com</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>10 × Chocolate chip cookies (box of 6), 3 × Greeting cards (set of 4)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>collected</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:05:00</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-05 15:05:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>OR-F1088AEA</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Mr Daniel Wong</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>daniel.wong@example.com</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>2 × Pineapple tarts (box of 10)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 10:40:00</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>OR-3B6FB7E1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Ms Priya Menon</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> +65 8100 0004</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>2 × Greeting cards (set of 4), 2 × Handmade tote bag</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 16:30:00</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="n"/>
+      <c r="N5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>OR-8E3DA6B2</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>FR-CCF4CA7D</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Charity bake sale</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Aunty Mei Ling</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>1 × Pineapple tarts (box of 10), 1 × Chocolate chip cookies (box of 6)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>unpaid</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:15:00</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="n"/>
+      <c r="N6" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Item ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Order ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Unit Price (SGD)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Line Total (SGD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>OI-2266E328</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>OR-8A99BCEC</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>PD-ADFCD451</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate chip cookies (box of 6)</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>OI-AC84D48C</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>OR-8A99BCEC</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>PD-D742F744</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Handmade tote bag</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>OI-F438D9D4</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OR-53D7A693</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>PD-ADFCD451</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate chip cookies (box of 6)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>OI-863D4635</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>OR-53D7A693</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CBBC0AF</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Greeting cards (set of 4)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>OI-8F47D1F2</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OR-F1088AEA</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CB6D8E4</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Pineapple tarts (box of 10)</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>OI-49158619</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>OR-3B6FB7E1</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CBBC0AF</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Greeting cards (set of 4)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>OI-FB2A8BAA</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>OR-3B6FB7E1</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>PD-D742F744</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Handmade tote bag</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>OI-0851C231</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>OR-8E3DA6B2</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>PD-5CB6D8E4</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Pineapple tarts (box of 10)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>OI-E1251A75</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>OR-8E3DA6B2</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>PD-ADFCD451</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate chip cookies (box of 6)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Outing ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Outing</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Singapore Zoo</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Meet at the school gate at 08:30. Bring a cap and water bottle.</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Assignment ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Outing ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Outing</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee ID</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee Name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer User ID</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer Name</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Boarded</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Boarded At</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>OA-8E77F23A</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Alex Tan Wei Ming</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>U-122C0943</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Aisha Rahman</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>OA-54393B1B</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Bea Lim Hui Min</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>U-6783B9DB</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Ben Koh</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>OA-27602AF4</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Chris Ng Jun Jie</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>U-DF9FA475</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Daniel Lee</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>OA-79A51919</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>T-0005</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Farid bin Rahman</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>U-784CE8AF</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Chloe Wong</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>OA-F2C8C256</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>T-0006</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Grace Chua Pei Shan</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>U-E4B78912</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Esther Ong</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>OA-DABE8046</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>OT-2462E215</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Zoo outing</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>T-0008</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Ivy Teo Xin Yi</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>U-3D8F31C7</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Faiz Hakim</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 14:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Trip ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Destination</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok cultural exchange</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok, Thailand</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Partner school visit, cooking class and city tour.</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>planning</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Participant ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Trip ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee ID</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee Name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer User ID</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer Name</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Medical Notes (for this trip)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Dietary Notes (for this trip)</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Registered By</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Registered At</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Updated By</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Updated At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TP-D99FB7C6</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok cultural exchange</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Alex Tan Wei Ming</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>U-122C0943</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Aisha Rahman</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Epilepsy care plan in the school office</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TP-7379D4DD</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok cultural exchange</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Bea Lim Hui Min</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>U-6783B9DB</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Ben Koh</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Peanut allergy; EpiPen in bag</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>TP-3FCE1ABB</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok cultural exchange</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>T-0004</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Dana Goh Li Ting</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>registered</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Needs a wheelchair-accessible room and transport.</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TP-6A0EA2F8</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Bangkok cultural exchange</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>T-0006</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Grace Chua Pei Shan</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>U-E4B78912</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Esther Ong</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>registered</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Type 1 diabetes: snack at 11am</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
         </is>
       </c>
     </row>
@@ -1690,6 +3884,665 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Item ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Trip ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Done By</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Done At</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Added By</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Added At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TL-9A523694</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Book flights</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:00:00</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TL-896FBB38</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Collect passport copies from caregivers</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>TL-051B67A9</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Buy travel insurance</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TL-DB4641C9</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Caregiver briefing session</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2026-11-28</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Expense ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Trip ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Amount (SGD)</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Paid By</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Added By</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Added At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TE-5BC1C218</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Flights deposit</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>MINDS office</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TE-D5357371</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>TR-965548DB</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Hotel deposit</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>680.5</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>MINDS office</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Visit ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee ID</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Trainee Name</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer User ID</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Volunteer Name</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Visit Date</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Daily Living</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Recorded By</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Recorded At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>HV-F7AAB94D</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Alex Tan Wei Ming</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>U-122C0943</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Aisha Rahman</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Mum is managing well; grandmother has moved in to help.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Dresses himself; needs reminders to drink water.</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Enjoys the Saturday music group.</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>No seizures this month.</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Share the picture schedule with the family.</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-20 18:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>HV-E5CC364D</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Bea Lim Hui Min</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>U-6783B9DB</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Ben Koh</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Dad works night shifts; aunt helps in the afternoons.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Wants to join an art class.</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Send details of the community art class to Mr Lim.</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03 19:30:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>HV-FF924B75</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>T-0005</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Farid bin Rahman</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>U-784CE8AF</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Chloe Wong</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Packs his own bag for the day centre now.</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Sleeping better since the new routine.</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Sarah Yeo</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:45:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4829,7 +7682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4845,6 +7698,8 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4911,6 +7766,16 @@
       <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Method</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Edited By</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Edited At</t>
         </is>
       </c>
     </row>

</xml_diff>